<commit_message>
Verify model-retirement kit and link it from its niche
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01DspfyLwNfeJ4CHdyACeRHQ
</commit_message>
<xml_diff>
--- a/kits/model-retirement/samples/compare/comparison.xlsx
+++ b/kits/model-retirement/samples/compare/comparison.xlsx
@@ -537,7 +537,7 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
+    <pageSetUpPr fitToPage="1"/>
   </sheetPr>
   <dimension ref="A1:D43"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
@@ -558,7 +558,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Generated 2026-10-07 10:12 by compare_runs.py. Test set: test_set.jsonl (10 cases).</t>
+          <t>Generated 2026-10-07 10:27 by compare_runs.py. Test set: test_set.jsonl (10 cases).</t>
         </is>
       </c>
     </row>
@@ -945,7 +945,7 @@
     <row r="30">
       <c r="A30" s="3" t="inlineStr">
         <is>
-          <t>Human grading (updates as you fill the Comparison sheet)</t>
+          <t>Human grading (updates as you grade)</t>
         </is>
       </c>
       <c r="B30" s="3" t="inlineStr">
@@ -1074,6 +1074,7 @@
     <mergeCell ref="A42:D42"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <pageSetup orientation="landscape" fitToHeight="0" fitToWidth="1"/>
 </worksheet>
 </file>
 
@@ -2210,6 +2211,7 @@
     </dataValidation>
   </dataValidations>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <pageSetup orientation="landscape"/>
 </worksheet>
 </file>
 
@@ -2543,5 +2545,6 @@
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <pageSetup orientation="landscape"/>
 </worksheet>
 </file>
</xml_diff>